<commit_message>
UV and .venv setup
</commit_message>
<xml_diff>
--- a/data/Business Case - Chatbot data - Raw Data.xlsx
+++ b/data/Business Case - Chatbot data - Raw Data.xlsx
@@ -1,23 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://adidasgroup-my.sharepoint.com/personal/valentina_ortiz_adidas_com/Documents/Documents/ME/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\restr\Desktop\TaskUs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FF26401-160F-4924-8E19-2512C2B7C3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF747B36-F3F8-497D-B03F-F041BFDB6EFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agent handled only volume" sheetId="1" r:id="rId1"/>
     <sheet name="Hybrid Handled only volume" sheetId="2" r:id="rId2"/>
     <sheet name="Bot only volume" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -514,9 +527,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,###"/>
     <numFmt numFmtId="165" formatCode="#,##0.##%"/>
+    <numFmt numFmtId="173" formatCode="#,##0.######%"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -547,10 +561,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -886,18 +901,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H185"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="36" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -920,7 +935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -943,7 +958,7 @@
         <v>0.17762548248004159</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -966,7 +981,7 @@
         <v>0.13095833029886766</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -989,7 +1004,7 @@
         <v>9.1646722902640115E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1012,7 +1027,7 @@
         <v>7.7390175362817462E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1035,7 +1050,7 @@
         <v>5.1988558599508294E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1058,7 +1073,7 @@
         <v>4.0667699640635553E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1081,7 +1096,7 @@
         <v>3.9783728399836266E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1104,7 +1119,7 @@
         <v>3.048445139790509E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1127,7 +1142,7 @@
         <v>2.8221786375290995E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1150,7 +1165,7 @@
         <v>2.6579407990396861E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1173,7 +1188,7 @@
         <v>1.8673892461885017E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1196,7 +1211,7 @@
         <v>1.721734894011346E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -1219,7 +1234,7 @@
         <v>1.4379600354593009E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1242,7 +1257,7 @@
         <v>1.426659266755901E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1265,7 +1280,7 @@
         <v>1.4163630108261362E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -1288,7 +1303,7 @@
         <v>1.408075780443643E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>4</v>
       </c>
@@ -1302,7 +1317,7 @@
         <v>1.3171673744296251E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>4</v>
       </c>
@@ -1316,7 +1331,15 @@
         <v>1.2732199405830695E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
+        <f>SUM(B2:B17)</f>
+        <v>398203</v>
+      </c>
+      <c r="C20" s="2">
+        <f>SUM(C2:C17)</f>
+        <v>1</v>
+      </c>
       <c r="E20" t="s">
         <v>10</v>
       </c>
@@ -1330,7 +1353,7 @@
         <v>1.0434376436139356E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>4</v>
       </c>
@@ -1344,7 +1367,15 @@
         <v>1.0431865154205267E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <f>SUM(G2:G185)</f>
+        <v>398203</v>
+      </c>
+      <c r="C22" s="3">
+        <f>SUM(H2:H185)</f>
+        <v>0.99999999999999956</v>
+      </c>
       <c r="E22" t="s">
         <v>8</v>
       </c>
@@ -1358,7 +1389,7 @@
         <v>1.0009969789278332E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
         <v>9</v>
       </c>
@@ -1372,7 +1403,7 @@
         <v>9.7839544152103324E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
         <v>3</v>
       </c>
@@ -1386,7 +1417,7 @@
         <v>9.4474426360424205E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
         <v>4</v>
       </c>
@@ -1400,7 +1431,7 @@
         <v>8.7116370293543743E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
         <v>11</v>
       </c>
@@ -1414,7 +1445,7 @@
         <v>8.478087809484107E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E27" t="s">
         <v>4</v>
       </c>
@@ -1428,7 +1459,7 @@
         <v>7.8301770704891725E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E28" t="s">
         <v>4</v>
       </c>
@@ -1442,7 +1473,7 @@
         <v>6.6498745614673926E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E29" t="s">
         <v>13</v>
       </c>
@@ -1456,7 +1487,7 @@
         <v>6.4816186718834367E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E30" t="s">
         <v>3</v>
       </c>
@@ -1470,7 +1501,7 @@
         <v>5.8814222896361908E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E31" t="s">
         <v>4</v>
       </c>
@@ -1484,7 +1515,7 @@
         <v>5.4595269247092564E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
         <v>4</v>
       </c>
@@ -1498,7 +1529,7 @@
         <v>5.414323849895656E-3</v>
       </c>
     </row>
-    <row r="33" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E33" t="s">
         <v>3</v>
       </c>
@@ -1512,7 +1543,7 @@
         <v>5.0351202778482328E-3</v>
       </c>
     </row>
-    <row r="34" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E34" t="s">
         <v>3</v>
       </c>
@@ -1526,7 +1557,7 @@
         <v>4.5077510716895657E-3</v>
       </c>
     </row>
-    <row r="35" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E35" t="s">
         <v>4</v>
       </c>
@@ -1540,7 +1571,7 @@
         <v>4.47510440654641E-3</v>
       </c>
     </row>
-    <row r="36" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E36" t="s">
         <v>4</v>
       </c>
@@ -1554,7 +1585,7 @@
         <v>4.173750574455742E-3</v>
       </c>
     </row>
-    <row r="37" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
         <v>4</v>
       </c>
@@ -1568,7 +1599,7 @@
         <v>3.7066521347152081E-3</v>
       </c>
     </row>
-    <row r="38" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E38" t="s">
         <v>4</v>
       </c>
@@ -1582,7 +1613,7 @@
         <v>3.4429675316358741E-3</v>
       </c>
     </row>
-    <row r="39" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E39" t="s">
         <v>4</v>
       </c>
@@ -1596,7 +1627,7 @@
         <v>3.3374936904041409E-3</v>
       </c>
     </row>
-    <row r="40" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E40" t="s">
         <v>8</v>
       </c>
@@ -1610,7 +1641,7 @@
         <v>3.2018844659633407E-3</v>
       </c>
     </row>
-    <row r="41" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E41" t="s">
         <v>12</v>
       </c>
@@ -1624,7 +1655,7 @@
         <v>3.1893280562928956E-3</v>
       </c>
     </row>
-    <row r="42" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>12</v>
       </c>
@@ -1638,7 +1669,7 @@
         <v>3.0060044751044064E-3</v>
       </c>
     </row>
-    <row r="43" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>4</v>
       </c>
@@ -1652,7 +1683,7 @@
         <v>2.9608014002908069E-3</v>
       </c>
     </row>
-    <row r="44" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>4</v>
       </c>
@@ -1666,7 +1697,7 @@
         <v>2.6544250043319612E-3</v>
       </c>
     </row>
-    <row r="45" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
         <v>4</v>
       </c>
@@ -1680,7 +1711,7 @@
         <v>2.2701988684163607E-3</v>
       </c>
     </row>
-    <row r="46" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
         <v>4</v>
       </c>
@@ -1694,7 +1725,7 @@
         <v>2.2425747671413828E-3</v>
       </c>
     </row>
-    <row r="47" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
         <v>4</v>
       </c>
@@ -1708,7 +1739,7 @@
         <v>2.1873265645914268E-3</v>
       </c>
     </row>
-    <row r="48" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
         <v>5</v>
       </c>
@@ -1722,7 +1753,7 @@
         <v>2.1170106704369381E-3</v>
       </c>
     </row>
-    <row r="49" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>8</v>
       </c>
@@ -1736,7 +1767,7 @@
         <v>1.7679424815985813E-3</v>
       </c>
     </row>
-    <row r="50" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>4</v>
       </c>
@@ -1750,7 +1781,7 @@
         <v>1.7528747899940482E-3</v>
       </c>
     </row>
-    <row r="51" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>3</v>
       </c>
@@ -1764,7 +1795,7 @@
         <v>1.6499122306964035E-3</v>
       </c>
     </row>
-    <row r="52" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>9</v>
       </c>
@@ -1778,7 +1809,7 @@
         <v>1.5795963365419143E-3</v>
       </c>
     </row>
-    <row r="53" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>9</v>
       </c>
@@ -1792,7 +1823,7 @@
         <v>1.2280168657694693E-3</v>
       </c>
     </row>
-    <row r="54" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>14</v>
       </c>
@@ -1806,7 +1837,7 @@
         <v>1.142633280010447E-3</v>
       </c>
     </row>
-    <row r="55" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>14</v>
       </c>
@@ -1820,7 +1851,7 @@
         <v>1.1401219980763581E-3</v>
       </c>
     </row>
-    <row r="56" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>9</v>
       </c>
@@ -1834,7 +1865,7 @@
         <v>1.0798512316582247E-3</v>
       </c>
     </row>
-    <row r="57" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>9</v>
       </c>
@@ -1848,7 +1879,7 @@
         <v>1.06729482198778E-3</v>
       </c>
     </row>
-    <row r="58" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>8</v>
       </c>
@@ -1862,7 +1893,7 @@
         <v>9.4675328915151322E-4</v>
       </c>
     </row>
-    <row r="59" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E59" t="s">
         <v>14</v>
       </c>
@@ -1876,7 +1907,7 @@
         <v>9.2917431561289092E-4</v>
       </c>
     </row>
-    <row r="60" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E60" t="s">
         <v>3</v>
       </c>
@@ -1890,7 +1921,7 @@
         <v>8.8145995886520199E-4</v>
       </c>
     </row>
-    <row r="61" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
         <v>4</v>
       </c>
@@ -1904,7 +1935,7 @@
         <v>7.1822663314942382E-4</v>
       </c>
     </row>
-    <row r="62" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
         <v>4</v>
       </c>
@@ -1918,7 +1949,7 @@
         <v>7.1822663314942382E-4</v>
       </c>
     </row>
-    <row r="63" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
         <v>9</v>
       </c>
@@ -1932,7 +1963,7 @@
         <v>5.8512869064271237E-4</v>
       </c>
     </row>
-    <row r="64" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E64" t="s">
         <v>9</v>
       </c>
@@ -1946,7 +1977,7 @@
         <v>5.7508356290635683E-4</v>
       </c>
     </row>
-    <row r="65" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
         <v>14</v>
       </c>
@@ -1960,7 +1991,7 @@
         <v>5.2988048809275668E-4</v>
       </c>
     </row>
-    <row r="66" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
         <v>12</v>
       </c>
@@ -1974,7 +2005,7 @@
         <v>4.9472254101551219E-4</v>
       </c>
     </row>
-    <row r="67" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
         <v>15</v>
       </c>
@@ -1988,7 +2019,7 @@
         <v>4.922112590814233E-4</v>
       </c>
     </row>
-    <row r="68" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
         <v>10</v>
       </c>
@@ -2002,7 +2033,7 @@
         <v>4.6960972167462323E-4</v>
       </c>
     </row>
-    <row r="69" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E69" t="s">
         <v>8</v>
       </c>
@@ -2016,7 +2047,7 @@
         <v>4.6207587587235657E-4</v>
       </c>
     </row>
-    <row r="70" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E70" t="s">
         <v>4</v>
       </c>
@@ -2030,7 +2061,7 @@
         <v>4.4198562039964533E-4</v>
       </c>
     </row>
-    <row r="71" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E71" t="s">
         <v>12</v>
       </c>
@@ -2044,7 +2075,7 @@
         <v>3.9929382752013418E-4</v>
       </c>
     </row>
-    <row r="72" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E72" t="s">
         <v>14</v>
       </c>
@@ -2058,7 +2089,7 @@
         <v>3.9427126365195635E-4</v>
       </c>
     </row>
-    <row r="73" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
         <v>16</v>
       </c>
@@ -2072,7 +2103,7 @@
         <v>3.515794707724452E-4</v>
       </c>
     </row>
-    <row r="74" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
         <v>10</v>
       </c>
@@ -2086,7 +2117,7 @@
         <v>3.4404562497017854E-4</v>
       </c>
     </row>
-    <row r="75" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E75" t="s">
         <v>6</v>
       </c>
@@ -2100,7 +2131,7 @@
         <v>3.2646665143155624E-4</v>
       </c>
     </row>
-    <row r="76" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E76" t="s">
         <v>4</v>
       </c>
@@ -2114,7 +2145,7 @@
         <v>3.2144408756337847E-4</v>
       </c>
     </row>
-    <row r="77" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>5</v>
       </c>
@@ -2128,7 +2159,7 @@
         <v>3.0135383209066734E-4</v>
       </c>
     </row>
-    <row r="78" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
         <v>5</v>
       </c>
@@ -2142,7 +2173,7 @@
         <v>2.7875229468386726E-4</v>
       </c>
     </row>
-    <row r="79" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E79" t="s">
         <v>9</v>
       </c>
@@ -2156,7 +2187,7 @@
         <v>2.5615075727706724E-4</v>
       </c>
     </row>
-    <row r="80" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E80" t="s">
         <v>15</v>
       </c>
@@ -2170,7 +2201,7 @@
         <v>2.4610562954071165E-4</v>
       </c>
     </row>
-    <row r="81" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E81" t="s">
         <v>5</v>
       </c>
@@ -2184,7 +2215,7 @@
         <v>2.3606050180435608E-4</v>
       </c>
     </row>
-    <row r="82" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E82" t="s">
         <v>9</v>
       </c>
@@ -2198,7 +2229,7 @@
         <v>2.235040921339116E-4</v>
       </c>
     </row>
-    <row r="83" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E83" t="s">
         <v>9</v>
       </c>
@@ -2212,7 +2243,7 @@
         <v>2.1597024633164492E-4</v>
       </c>
     </row>
-    <row r="84" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E84" t="s">
         <v>3</v>
       </c>
@@ -2226,7 +2257,7 @@
         <v>2.1094768246346713E-4</v>
       </c>
     </row>
-    <row r="85" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E85" t="s">
         <v>4</v>
       </c>
@@ -2240,7 +2271,7 @@
         <v>1.9587999085893379E-4</v>
       </c>
     </row>
-    <row r="86" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E86" t="s">
         <v>3</v>
       </c>
@@ -2254,7 +2285,7 @@
         <v>1.9587999085893379E-4</v>
       </c>
     </row>
-    <row r="87" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E87" t="s">
         <v>3</v>
       </c>
@@ -2268,7 +2299,7 @@
         <v>1.9085742699075596E-4</v>
       </c>
     </row>
-    <row r="88" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E88" t="s">
         <v>14</v>
       </c>
@@ -2282,7 +2313,7 @@
         <v>1.8834614505666711E-4</v>
       </c>
     </row>
-    <row r="89" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E89" t="s">
         <v>6</v>
       </c>
@@ -2296,7 +2327,7 @@
         <v>1.5821076184760032E-4</v>
       </c>
     </row>
-    <row r="90" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E90" t="s">
         <v>14</v>
       </c>
@@ -2310,7 +2341,7 @@
         <v>1.4816563411124476E-4</v>
       </c>
     </row>
-    <row r="91" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E91" t="s">
         <v>12</v>
       </c>
@@ -2324,7 +2355,7 @@
         <v>1.4816563411124476E-4</v>
       </c>
     </row>
-    <row r="92" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E92" t="s">
         <v>15</v>
       </c>
@@ -2338,7 +2369,7 @@
         <v>1.4565435217715587E-4</v>
       </c>
     </row>
-    <row r="93" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E93" t="s">
         <v>4</v>
       </c>
@@ -2352,7 +2383,7 @@
         <v>1.3309794250671139E-4</v>
       </c>
     </row>
-    <row r="94" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E94" t="s">
         <v>15</v>
       </c>
@@ -2366,7 +2397,7 @@
         <v>1.3058666057262251E-4</v>
       </c>
     </row>
-    <row r="95" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E95" t="s">
         <v>3</v>
       </c>
@@ -2380,7 +2411,7 @@
         <v>1.2305281477035583E-4</v>
       </c>
     </row>
-    <row r="96" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E96" t="s">
         <v>14</v>
       </c>
@@ -2394,7 +2425,7 @@
         <v>1.1300768703400024E-4</v>
       </c>
     </row>
-    <row r="97" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E97" t="s">
         <v>9</v>
       </c>
@@ -2408,7 +2439,7 @@
         <v>1.0547384123173356E-4</v>
       </c>
     </row>
-    <row r="98" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E98" t="s">
         <v>6</v>
       </c>
@@ -2422,7 +2453,7 @@
         <v>9.7939995429466894E-5</v>
       </c>
     </row>
-    <row r="99" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E99" t="s">
         <v>14</v>
       </c>
@@ -2436,7 +2467,7 @@
         <v>9.2917431561289097E-5</v>
       </c>
     </row>
-    <row r="100" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E100" t="s">
         <v>14</v>
       </c>
@@ -2450,7 +2481,7 @@
         <v>9.2917431561289097E-5</v>
       </c>
     </row>
-    <row r="101" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E101" t="s">
         <v>12</v>
       </c>
@@ -2464,7 +2495,7 @@
         <v>9.0406149627200212E-5</v>
       </c>
     </row>
-    <row r="102" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E102" t="s">
         <v>9</v>
       </c>
@@ -2478,7 +2509,7 @@
         <v>8.5383585759022415E-5</v>
       </c>
     </row>
-    <row r="103" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E103" t="s">
         <v>4</v>
       </c>
@@ -2492,7 +2523,7 @@
         <v>7.7849739956755719E-5</v>
       </c>
     </row>
-    <row r="104" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E104" t="s">
         <v>15</v>
       </c>
@@ -2506,7 +2537,7 @@
         <v>7.5338458022666834E-5</v>
       </c>
     </row>
-    <row r="105" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E105" t="s">
         <v>15</v>
       </c>
@@ -2520,7 +2551,7 @@
         <v>6.2782048352222355E-5</v>
       </c>
     </row>
-    <row r="106" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E106" t="s">
         <v>6</v>
       </c>
@@ -2534,7 +2565,7 @@
         <v>5.7759484484044572E-5</v>
       </c>
     </row>
-    <row r="107" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E107" t="s">
         <v>14</v>
       </c>
@@ -2548,7 +2579,7 @@
         <v>5.5248202549955666E-5</v>
       </c>
     </row>
-    <row r="108" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
         <v>3</v>
       </c>
@@ -2562,7 +2593,7 @@
         <v>5.5248202549955666E-5</v>
       </c>
     </row>
-    <row r="109" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E109" t="s">
         <v>6</v>
       </c>
@@ -2576,7 +2607,7 @@
         <v>5.2736920615866781E-5</v>
       </c>
     </row>
-    <row r="110" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E110" t="s">
         <v>3</v>
       </c>
@@ -2590,7 +2621,7 @@
         <v>4.5203074813600106E-5</v>
       </c>
     </row>
-    <row r="111" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
         <v>15</v>
       </c>
@@ -2604,7 +2635,7 @@
         <v>4.2691792879511207E-5</v>
       </c>
     </row>
-    <row r="112" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E112" t="s">
         <v>9</v>
       </c>
@@ -2618,7 +2649,7 @@
         <v>4.0180510945422309E-5</v>
       </c>
     </row>
-    <row r="113" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E113" t="s">
         <v>17</v>
       </c>
@@ -2632,7 +2663,7 @@
         <v>4.0180510945422309E-5</v>
       </c>
     </row>
-    <row r="114" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E114" t="s">
         <v>4</v>
       </c>
@@ -2646,7 +2677,7 @@
         <v>3.5157947077244519E-5</v>
       </c>
     </row>
-    <row r="115" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="115" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E115" t="s">
         <v>3</v>
       </c>
@@ -2660,7 +2691,7 @@
         <v>3.5157947077244519E-5</v>
       </c>
     </row>
-    <row r="116" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
         <v>15</v>
       </c>
@@ -2674,7 +2705,7 @@
         <v>3.5157947077244519E-5</v>
       </c>
     </row>
-    <row r="117" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
         <v>15</v>
       </c>
@@ -2688,7 +2719,7 @@
         <v>3.5157947077244519E-5</v>
       </c>
     </row>
-    <row r="118" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E118" t="s">
         <v>15</v>
       </c>
@@ -2702,7 +2733,7 @@
         <v>3.2646665143155627E-5</v>
       </c>
     </row>
-    <row r="119" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E119" t="s">
         <v>15</v>
       </c>
@@ -2716,7 +2747,7 @@
         <v>3.2646665143155627E-5</v>
       </c>
     </row>
-    <row r="120" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E120" t="s">
         <v>3</v>
       </c>
@@ -2730,7 +2761,7 @@
         <v>3.0135383209066732E-5</v>
       </c>
     </row>
-    <row r="121" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E121" t="s">
         <v>4</v>
       </c>
@@ -2744,7 +2775,7 @@
         <v>2.7624101274977833E-5</v>
       </c>
     </row>
-    <row r="122" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E122" t="s">
         <v>9</v>
       </c>
@@ -2758,7 +2789,7 @@
         <v>2.0090255472711154E-5</v>
       </c>
     </row>
-    <row r="123" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E123" t="s">
         <v>15</v>
       </c>
@@ -2772,7 +2803,7 @@
         <v>1.7578973538622259E-5</v>
       </c>
     </row>
-    <row r="124" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
         <v>15</v>
       </c>
@@ -2786,7 +2817,7 @@
         <v>1.7578973538622259E-5</v>
       </c>
     </row>
-    <row r="125" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E125" t="s">
         <v>15</v>
       </c>
@@ -2800,7 +2831,7 @@
         <v>1.5067691604533366E-5</v>
       </c>
     </row>
-    <row r="126" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E126" t="s">
         <v>15</v>
       </c>
@@ -2814,7 +2845,7 @@
         <v>1.5067691604533366E-5</v>
       </c>
     </row>
-    <row r="127" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E127" t="s">
         <v>15</v>
       </c>
@@ -2828,7 +2859,7 @@
         <v>1.5067691604533366E-5</v>
       </c>
     </row>
-    <row r="128" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E128" t="s">
         <v>14</v>
       </c>
@@ -2842,7 +2873,7 @@
         <v>1.2556409670444472E-5</v>
       </c>
     </row>
-    <row r="129" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E129" t="s">
         <v>4</v>
       </c>
@@ -2856,7 +2887,7 @@
         <v>1.2556409670444472E-5</v>
       </c>
     </row>
-    <row r="130" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E130" t="s">
         <v>12</v>
       </c>
@@ -2870,7 +2901,7 @@
         <v>1.2556409670444472E-5</v>
       </c>
     </row>
-    <row r="131" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E131" t="s">
         <v>15</v>
       </c>
@@ -2884,7 +2915,7 @@
         <v>1.2556409670444472E-5</v>
       </c>
     </row>
-    <row r="132" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E132" t="s">
         <v>10</v>
       </c>
@@ -2898,7 +2929,7 @@
         <v>1.0045127736355577E-5</v>
       </c>
     </row>
-    <row r="133" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E133" t="s">
         <v>4</v>
       </c>
@@ -2912,7 +2943,7 @@
         <v>1.0045127736355577E-5</v>
       </c>
     </row>
-    <row r="134" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E134" t="s">
         <v>9</v>
       </c>
@@ -2926,7 +2957,7 @@
         <v>1.0045127736355577E-5</v>
       </c>
     </row>
-    <row r="135" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E135" t="s">
         <v>15</v>
       </c>
@@ -2940,7 +2971,7 @@
         <v>1.0045127736355577E-5</v>
       </c>
     </row>
-    <row r="136" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E136" t="s">
         <v>14</v>
       </c>
@@ -2954,7 +2985,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="137" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E137" t="s">
         <v>10</v>
       </c>
@@ -2968,7 +2999,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="138" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="138" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E138" t="s">
         <v>10</v>
       </c>
@@ -2982,7 +3013,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="139" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E139" t="s">
         <v>4</v>
       </c>
@@ -2996,7 +3027,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="140" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E140" t="s">
         <v>8</v>
       </c>
@@ -3010,7 +3041,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="141" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E141" t="s">
         <v>3</v>
       </c>
@@ -3024,7 +3055,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="142" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E142" t="s">
         <v>3</v>
       </c>
@@ -3038,7 +3069,7 @@
         <v>7.5338458022666829E-6</v>
       </c>
     </row>
-    <row r="143" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="143" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E143" t="s">
         <v>14</v>
       </c>
@@ -3052,7 +3083,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="144" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E144" t="s">
         <v>5</v>
       </c>
@@ -3066,7 +3097,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="145" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E145" t="s">
         <v>10</v>
       </c>
@@ -3080,7 +3111,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="146" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E146" t="s">
         <v>4</v>
       </c>
@@ -3094,7 +3125,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="147" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E147" t="s">
         <v>18</v>
       </c>
@@ -3108,7 +3139,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="148" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E148" t="s">
         <v>12</v>
       </c>
@@ -3122,7 +3153,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="149" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E149" t="s">
         <v>15</v>
       </c>
@@ -3136,7 +3167,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="150" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E150" t="s">
         <v>15</v>
       </c>
@@ -3150,7 +3181,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="151" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E151" t="s">
         <v>15</v>
       </c>
@@ -3164,7 +3195,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="152" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E152" t="s">
         <v>15</v>
       </c>
@@ -3178,7 +3209,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="153" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E153" t="s">
         <v>7</v>
       </c>
@@ -3192,7 +3223,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="154" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E154" t="s">
         <v>7</v>
       </c>
@@ -3206,7 +3237,7 @@
         <v>5.0225638681777886E-6</v>
       </c>
     </row>
-    <row r="155" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E155" t="s">
         <v>5</v>
       </c>
@@ -3220,7 +3251,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="156" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E156" t="s">
         <v>5</v>
       </c>
@@ -3234,7 +3265,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="157" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E157" t="s">
         <v>5</v>
       </c>
@@ -3248,7 +3279,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="158" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E158" t="s">
         <v>5</v>
       </c>
@@ -3262,7 +3293,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="159" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E159" t="s">
         <v>5</v>
       </c>
@@ -3276,7 +3307,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="160" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E160" t="s">
         <v>5</v>
       </c>
@@ -3290,7 +3321,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="161" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E161" t="s">
         <v>10</v>
       </c>
@@ -3304,7 +3335,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="162" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="162" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E162" t="s">
         <v>10</v>
       </c>
@@ -3318,7 +3349,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="163" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E163" t="s">
         <v>10</v>
       </c>
@@ -3332,7 +3363,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="164" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E164" t="s">
         <v>18</v>
       </c>
@@ -3346,7 +3377,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="165" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E165" t="s">
         <v>18</v>
       </c>
@@ -3360,7 +3391,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="166" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
         <v>8</v>
       </c>
@@ -3374,7 +3405,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="167" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E167" t="s">
         <v>8</v>
       </c>
@@ -3388,7 +3419,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="168" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E168" t="s">
         <v>12</v>
       </c>
@@ -3402,7 +3433,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="169" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E169" t="s">
         <v>3</v>
       </c>
@@ -3416,7 +3447,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="170" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E170" t="s">
         <v>3</v>
       </c>
@@ -3430,7 +3461,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="171" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E171" t="s">
         <v>3</v>
       </c>
@@ -3444,7 +3475,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="172" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E172" t="s">
         <v>3</v>
       </c>
@@ -3458,7 +3489,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="173" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E173" t="s">
         <v>3</v>
       </c>
@@ -3472,7 +3503,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="174" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E174" t="s">
         <v>3</v>
       </c>
@@ -3486,7 +3517,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="175" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E175" t="s">
         <v>3</v>
       </c>
@@ -3500,7 +3531,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="176" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E176" t="s">
         <v>15</v>
       </c>
@@ -3514,7 +3545,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="177" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E177" t="s">
         <v>15</v>
       </c>
@@ -3528,7 +3559,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="178" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E178" t="s">
         <v>7</v>
       </c>
@@ -3542,7 +3573,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="179" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E179" t="s">
         <v>7</v>
       </c>
@@ -3556,7 +3587,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="180" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E180" t="s">
         <v>7</v>
       </c>
@@ -3570,7 +3601,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="181" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E181" t="s">
         <v>7</v>
       </c>
@@ -3584,7 +3615,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="182" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E182" t="s">
         <v>7</v>
       </c>
@@ -3598,7 +3629,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="183" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E183" t="s">
         <v>7</v>
       </c>
@@ -3612,7 +3643,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="184" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E184" t="s">
         <v>6</v>
       </c>
@@ -3626,7 +3657,7 @@
         <v>2.5112819340888943E-6</v>
       </c>
     </row>
-    <row r="185" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E185" t="s">
         <v>6</v>
       </c>
@@ -3648,18 +3679,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26EF6205-7A82-4AA6-8B49-FF192981C801}">
   <dimension ref="A1:H209"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="36" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3682,7 +3713,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3705,7 +3736,7 @@
         <v>9.6400861134790711E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3728,7 +3759,7 @@
         <v>7.4305384982156011E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -3751,7 +3782,7 @@
         <v>6.5372556385545649E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3774,7 +3805,7 @@
         <v>5.410267154065105E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3797,7 +3828,7 @@
         <v>5.0671136091083785E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3820,7 +3851,7 @@
         <v>5.0154599702359449E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -3843,7 +3874,7 @@
         <v>4.8825331233474448E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -3866,7 +3897,7 @@
         <v>4.2493245293378223E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -3889,7 +3920,7 @@
         <v>3.7335105691291844E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -3912,7 +3943,7 @@
         <v>2.9612344858476254E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -3935,7 +3966,7 @@
         <v>2.4194130990738468E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -3958,7 +3989,7 @@
         <v>2.2196616144832468E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -3981,7 +4012,7 @@
         <v>1.8508618572192281E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -4004,7 +4035,7 @@
         <v>1.7815087197121843E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -4027,7 +4058,7 @@
         <v>1.7609195070147809E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -4050,7 +4081,7 @@
         <v>1.747554579474361E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -4073,7 +4104,7 @@
         <v>1.5669474505497681E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -4096,7 +4127,7 @@
         <v>1.5463582378523643E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -4119,7 +4150,7 @@
         <v>1.5044573839418589E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>12</v>
       </c>
@@ -4133,7 +4164,7 @@
         <v>1.2675008307927931E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
         <v>12</v>
       </c>
@@ -4147,7 +4178,7 @@
         <v>1.2620826169250553E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
         <v>8</v>
       </c>
@@ -4161,7 +4192,7 @@
         <v>1.1605814104694341E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
         <v>21</v>
       </c>
@@ -4175,7 +4206,7 @@
         <v>1.1092889858548496E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
         <v>10</v>
       </c>
@@ -4189,7 +4220,7 @@
         <v>1.03812977705856E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
         <v>4</v>
       </c>
@@ -4203,7 +4234,7 @@
         <v>1.0211527069396481E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E27" t="s">
         <v>3</v>
       </c>
@@ -4217,7 +4248,7 @@
         <v>1.0092326364306252E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E28" t="s">
         <v>4</v>
       </c>
@@ -4231,7 +4262,7 @@
         <v>9.7600092470850001E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E29" t="s">
         <v>3</v>
       </c>
@@ -4245,7 +4276,7 @@
         <v>9.2326364306251889E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E30" t="s">
         <v>12</v>
       </c>
@@ -4259,7 +4290,7 @@
         <v>8.6474693329095086E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E31" t="s">
         <v>4</v>
       </c>
@@ -4273,7 +4304,7 @@
         <v>8.0081200965164499E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
         <v>9</v>
       </c>
@@ -4287,7 +4318,7 @@
         <v>7.646905838667264E-3</v>
       </c>
     </row>
-    <row r="33" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E33" t="s">
         <v>4</v>
       </c>
@@ -4301,7 +4332,7 @@
         <v>7.3904437155943416E-3</v>
       </c>
     </row>
-    <row r="34" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E34" t="s">
         <v>3</v>
       </c>
@@ -4315,7 +4346,7 @@
         <v>7.2459580124546678E-3</v>
       </c>
     </row>
-    <row r="35" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E35" t="s">
         <v>4</v>
       </c>
@@ -4329,7 +4360,7 @@
         <v>7.242345869876177E-3</v>
       </c>
     </row>
-    <row r="36" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E36" t="s">
         <v>4</v>
       </c>
@@ -4343,7 +4374,7 @@
         <v>6.9317016081258762E-3</v>
       </c>
     </row>
-    <row r="37" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
         <v>8</v>
       </c>
@@ -4357,7 +4388,7 @@
         <v>6.7294216237303315E-3</v>
       </c>
     </row>
-    <row r="38" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E38" t="s">
         <v>4</v>
       </c>
@@ -4371,7 +4402,7 @@
         <v>6.2562309459478996E-3</v>
       </c>
     </row>
-    <row r="39" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E39" t="s">
         <v>3</v>
       </c>
@@ -4385,7 +4416,7 @@
         <v>5.8661195474707774E-3</v>
       </c>
     </row>
-    <row r="40" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E40" t="s">
         <v>9</v>
       </c>
@@ -4399,7 +4430,7 @@
         <v>5.5410267154065111E-3</v>
       </c>
     </row>
-    <row r="41" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E41" t="s">
         <v>4</v>
       </c>
@@ -4413,7 +4444,7 @@
         <v>5.4976810044646083E-3</v>
       </c>
     </row>
-    <row r="42" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>3</v>
       </c>
@@ -4427,7 +4458,7 @@
         <v>4.7535796332952851E-3</v>
       </c>
     </row>
-    <row r="43" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>4</v>
       </c>
@@ -4441,7 +4472,7 @@
         <v>4.4393232289664936E-3</v>
       </c>
     </row>
-    <row r="44" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>4</v>
       </c>
@@ -4455,7 +4486,7 @@
         <v>4.4068139457600674E-3</v>
       </c>
     </row>
-    <row r="45" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
         <v>13</v>
       </c>
@@ -4469,7 +4500,7 @@
         <v>4.3165103812977702E-3</v>
       </c>
     </row>
-    <row r="46" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
         <v>4</v>
       </c>
@@ -4483,7 +4514,7 @@
         <v>4.2912253832483272E-3</v>
       </c>
     </row>
-    <row r="47" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
         <v>4</v>
       </c>
@@ -4497,7 +4528,7 @@
         <v>3.9589082660270768E-3</v>
       </c>
     </row>
-    <row r="48" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
         <v>4</v>
       </c>
@@ -4511,7 +4542,7 @@
         <v>3.8144225628874025E-3</v>
       </c>
     </row>
-    <row r="49" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>20</v>
       </c>
@@ -4525,7 +4556,7 @@
         <v>3.6554882894337605E-3</v>
       </c>
     </row>
-    <row r="50" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>9</v>
       </c>
@@ -4539,7 +4570,7 @@
         <v>3.2039704671222784E-3</v>
       </c>
     </row>
-    <row r="51" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>8</v>
       </c>
@@ -4553,7 +4584,7 @@
         <v>3.055872621404112E-3</v>
       </c>
     </row>
-    <row r="52" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>11</v>
       </c>
@@ -4567,7 +4598,7 @@
         <v>2.9149990608429298E-3</v>
       </c>
     </row>
-    <row r="53" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>12</v>
       </c>
@@ -4581,7 +4612,7 @@
         <v>2.712719076447385E-3</v>
       </c>
     </row>
-    <row r="54" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>4</v>
       </c>
@@ -4595,7 +4626,7 @@
         <v>2.6946583635549261E-3</v>
       </c>
     </row>
-    <row r="55" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>4</v>
       </c>
@@ -4609,7 +4640,7 @@
         <v>2.6765976506624668E-3</v>
       </c>
     </row>
-    <row r="56" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>14</v>
       </c>
@@ -4623,7 +4654,7 @@
         <v>2.5862940862001705E-3</v>
       </c>
     </row>
-    <row r="57" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>4</v>
       </c>
@@ -4637,7 +4668,7 @@
         <v>2.5429483752582682E-3</v>
       </c>
     </row>
-    <row r="58" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>9</v>
       </c>
@@ -4651,7 +4682,7 @@
         <v>2.5393362326797762E-3</v>
       </c>
     </row>
-    <row r="59" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E59" t="s">
         <v>9</v>
       </c>
@@ -4665,7 +4696,7 @@
         <v>2.4237476701680369E-3</v>
       </c>
     </row>
-    <row r="60" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E60" t="s">
         <v>8</v>
       </c>
@@ -4679,7 +4710,7 @@
         <v>1.9722298478565548E-3</v>
       </c>
     </row>
-    <row r="61" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
         <v>4</v>
       </c>
@@ -4693,7 +4724,7 @@
         <v>1.9686177052780627E-3</v>
       </c>
     </row>
-    <row r="62" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
         <v>4</v>
       </c>
@@ -4707,7 +4738,7 @@
         <v>1.9072112814437013E-3</v>
       </c>
     </row>
-    <row r="63" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
         <v>14</v>
       </c>
@@ -4721,7 +4752,7 @@
         <v>1.6760341564202221E-3</v>
       </c>
     </row>
-    <row r="64" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E64" t="s">
         <v>14</v>
       </c>
@@ -4735,7 +4766,7 @@
         <v>1.6146277325858607E-3</v>
       </c>
     </row>
-    <row r="65" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
         <v>12</v>
       </c>
@@ -4749,7 +4780,7 @@
         <v>1.5243241681235642E-3</v>
       </c>
     </row>
-    <row r="66" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
         <v>9</v>
       </c>
@@ -4763,7 +4794,7 @@
         <v>1.5134877403880887E-3</v>
       </c>
     </row>
-    <row r="67" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
         <v>4</v>
       </c>
@@ -4777,7 +4808,7 @@
         <v>1.4304084610827759E-3</v>
       </c>
     </row>
-    <row r="68" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
         <v>9</v>
       </c>
@@ -4791,7 +4822,7 @@
         <v>1.4304084610827759E-3</v>
       </c>
     </row>
-    <row r="69" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E69" t="s">
         <v>10</v>
       </c>
@@ -4805,7 +4836,7 @@
         <v>1.4015113204548411E-3</v>
       </c>
     </row>
-    <row r="70" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E70" t="s">
         <v>14</v>
       </c>
@@ -4819,7 +4850,7 @@
         <v>1.3401048966204796E-3</v>
       </c>
     </row>
-    <row r="71" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E71" t="s">
         <v>4</v>
       </c>
@@ -4833,7 +4864,7 @@
         <v>1.3003713282570689E-3</v>
       </c>
     </row>
-    <row r="72" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E72" t="s">
         <v>14</v>
       </c>
@@ -4847,7 +4878,7 @@
         <v>1.2750863302076259E-3</v>
       </c>
     </row>
-    <row r="73" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
         <v>9</v>
       </c>
@@ -4861,7 +4892,7 @@
         <v>1.2606377598936586E-3</v>
       </c>
     </row>
-    <row r="74" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
         <v>6</v>
       </c>
@@ -4875,7 +4906,7 @@
         <v>1.1631099102743783E-3</v>
       </c>
     </row>
-    <row r="75" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E75" t="s">
         <v>12</v>
       </c>
@@ -4889,7 +4920,7 @@
         <v>1.148661339960411E-3</v>
       </c>
     </row>
-    <row r="76" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E76" t="s">
         <v>9</v>
       </c>
@@ -4903,7 +4934,7 @@
         <v>1.1053156290185087E-3</v>
       </c>
     </row>
-    <row r="77" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>8</v>
       </c>
@@ -4917,7 +4948,7 @@
         <v>1.0402970626056552E-3</v>
       </c>
     </row>
-    <row r="78" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
         <v>3</v>
       </c>
@@ -4931,7 +4962,7 @@
         <v>1.0150120645562122E-3</v>
       </c>
     </row>
-    <row r="79" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E79" t="s">
         <v>3</v>
       </c>
@@ -4945,7 +4976,7 @@
         <v>1.0041756368207365E-3</v>
       </c>
     </row>
-    <row r="80" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E80" t="s">
         <v>3</v>
       </c>
@@ -4959,7 +4990,7 @@
         <v>9.7527849619280169E-4</v>
       </c>
     </row>
-    <row r="81" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E81" t="s">
         <v>8</v>
       </c>
@@ -4973,7 +5004,7 @@
         <v>8.1995636531765183E-4</v>
       </c>
     </row>
-    <row r="82" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E82" t="s">
         <v>14</v>
       </c>
@@ -4987,7 +5018,7 @@
         <v>7.2604065827686364E-4</v>
       </c>
     </row>
-    <row r="83" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E83" t="s">
         <v>4</v>
       </c>
@@ -5001,7 +5032,7 @@
         <v>7.1520423054138795E-4</v>
       </c>
     </row>
-    <row r="84" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E84" t="s">
         <v>4</v>
       </c>
@@ -5015,7 +5046,7 @@
         <v>6.826949473349612E-4</v>
       </c>
     </row>
-    <row r="85" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E85" t="s">
         <v>4</v>
       </c>
@@ -5029,7 +5060,7 @@
         <v>6.7185851959948551E-4</v>
       </c>
     </row>
-    <row r="86" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E86" t="s">
         <v>4</v>
       </c>
@@ -5043,7 +5074,7 @@
         <v>6.5018566412853446E-4</v>
       </c>
     </row>
-    <row r="87" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E87" t="s">
         <v>6</v>
       </c>
@@ -5057,7 +5088,7 @@
         <v>6.1767638092210771E-4</v>
       </c>
     </row>
-    <row r="88" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E88" t="s">
         <v>9</v>
       </c>
@@ -5071,7 +5102,7 @@
         <v>5.9239138287266473E-4</v>
       </c>
     </row>
-    <row r="89" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E89" t="s">
         <v>5</v>
       </c>
@@ -5085,7 +5116,7 @@
         <v>5.887792402941729E-4</v>
       </c>
     </row>
-    <row r="90" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E90" t="s">
         <v>14</v>
       </c>
@@ -5099,7 +5130,7 @@
         <v>4.6596639262544973E-4</v>
       </c>
     </row>
-    <row r="91" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E91" t="s">
         <v>13</v>
       </c>
@@ -5113,7 +5144,7 @@
         <v>4.5151782231148227E-4</v>
       </c>
     </row>
-    <row r="92" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E92" t="s">
         <v>6</v>
       </c>
@@ -5127,7 +5158,7 @@
         <v>4.479056797329904E-4</v>
       </c>
     </row>
-    <row r="93" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E93" t="s">
         <v>3</v>
       </c>
@@ -5141,7 +5172,7 @@
         <v>4.1539639652656371E-4</v>
       </c>
     </row>
-    <row r="94" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E94" t="s">
         <v>4</v>
       </c>
@@ -5155,7 +5186,7 @@
         <v>3.7566282816315326E-4</v>
       </c>
     </row>
-    <row r="95" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E95" t="s">
         <v>3</v>
       </c>
@@ -5169,7 +5200,7 @@
         <v>3.7566282816315326E-4</v>
       </c>
     </row>
-    <row r="96" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E96" t="s">
         <v>9</v>
       </c>
@@ -5183,7 +5214,7 @@
         <v>3.6843854300616955E-4</v>
       </c>
     </row>
-    <row r="97" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E97" t="s">
         <v>6</v>
       </c>
@@ -5197,7 +5228,7 @@
         <v>3.612142578491858E-4</v>
       </c>
     </row>
-    <row r="98" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E98" t="s">
         <v>14</v>
       </c>
@@ -5211,7 +5242,7 @@
         <v>3.5037783011371027E-4</v>
       </c>
     </row>
-    <row r="99" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E99" t="s">
         <v>5</v>
       </c>
@@ -5225,7 +5256,7 @@
         <v>3.3954140237823469E-4</v>
       </c>
     </row>
-    <row r="100" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E100" t="s">
         <v>7</v>
       </c>
@@ -5239,7 +5270,7 @@
         <v>3.3954140237823469E-4</v>
       </c>
     </row>
-    <row r="101" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E101" t="s">
         <v>3</v>
       </c>
@@ -5253,7 +5284,7 @@
         <v>2.9258354885784054E-4</v>
       </c>
     </row>
-    <row r="102" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E102" t="s">
         <v>9</v>
       </c>
@@ -5267,7 +5298,7 @@
         <v>2.8535926370085678E-4</v>
       </c>
     </row>
-    <row r="103" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E103" t="s">
         <v>10</v>
       </c>
@@ -5281,7 +5312,7 @@
         <v>2.7813497854387308E-4</v>
       </c>
     </row>
-    <row r="104" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E104" t="s">
         <v>14</v>
       </c>
@@ -5295,7 +5326,7 @@
         <v>2.3840141018046266E-4</v>
       </c>
     </row>
-    <row r="105" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E105" t="s">
         <v>4</v>
       </c>
@@ -5309,7 +5340,7 @@
         <v>2.3840141018046266E-4</v>
       </c>
     </row>
-    <row r="106" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E106" t="s">
         <v>9</v>
       </c>
@@ -5323,7 +5354,7 @@
         <v>2.1311641213101967E-4</v>
       </c>
     </row>
-    <row r="107" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E107" t="s">
         <v>6</v>
       </c>
@@ -5337,7 +5368,7 @@
         <v>2.1311641213101967E-4</v>
       </c>
     </row>
-    <row r="108" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
         <v>4</v>
       </c>
@@ -5351,7 +5382,7 @@
         <v>1.9866784181705221E-4</v>
       </c>
     </row>
-    <row r="109" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E109" t="s">
         <v>12</v>
       </c>
@@ -5365,7 +5396,7 @@
         <v>1.9866784181705221E-4</v>
       </c>
     </row>
-    <row r="110" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E110" t="s">
         <v>6</v>
       </c>
@@ -5379,7 +5410,7 @@
         <v>1.9866784181705221E-4</v>
       </c>
     </row>
-    <row r="111" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
         <v>14</v>
       </c>
@@ -5393,7 +5424,7 @@
         <v>1.9505569923856033E-4</v>
       </c>
     </row>
-    <row r="112" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E112" t="s">
         <v>3</v>
       </c>
@@ -5407,7 +5438,7 @@
         <v>1.9144355666006848E-4</v>
       </c>
     </row>
-    <row r="113" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E113" t="s">
         <v>12</v>
       </c>
@@ -5421,7 +5452,7 @@
         <v>1.733828437676092E-4</v>
       </c>
     </row>
-    <row r="114" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E114" t="s">
         <v>5</v>
       </c>
@@ -5435,7 +5466,7 @@
         <v>1.6615855861062547E-4</v>
       </c>
     </row>
-    <row r="115" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="115" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E115" t="s">
         <v>4</v>
       </c>
@@ -5449,7 +5480,7 @@
         <v>1.6254641603213361E-4</v>
       </c>
     </row>
-    <row r="116" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
         <v>6</v>
       </c>
@@ -5463,7 +5494,7 @@
         <v>1.6254641603213361E-4</v>
       </c>
     </row>
-    <row r="117" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
         <v>12</v>
       </c>
@@ -5477,7 +5508,7 @@
         <v>1.5170998829665803E-4</v>
       </c>
     </row>
-    <row r="118" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E118" t="s">
         <v>4</v>
       </c>
@@ -5491,7 +5522,7 @@
         <v>1.4809784571816618E-4</v>
       </c>
     </row>
-    <row r="119" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E119" t="s">
         <v>9</v>
       </c>
@@ -5505,7 +5536,7 @@
         <v>1.372614179826906E-4</v>
       </c>
     </row>
-    <row r="120" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E120" t="s">
         <v>3</v>
       </c>
@@ -5519,7 +5550,7 @@
         <v>1.2642499024721505E-4</v>
       </c>
     </row>
-    <row r="121" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E121" t="s">
         <v>3</v>
       </c>
@@ -5533,7 +5564,7 @@
         <v>1.1558856251173945E-4</v>
       </c>
     </row>
-    <row r="122" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E122" t="s">
         <v>9</v>
       </c>
@@ -5547,7 +5578,7 @@
         <v>1.0113999219777203E-4</v>
       </c>
     </row>
-    <row r="123" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E123" t="s">
         <v>4</v>
       </c>
@@ -5561,7 +5592,7 @@
         <v>9.3915707040788314E-5</v>
       </c>
     </row>
-    <row r="124" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
         <v>4</v>
       </c>
@@ -5575,7 +5606,7 @@
         <v>8.6691421883804598E-5</v>
       </c>
     </row>
-    <row r="125" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E125" t="s">
         <v>5</v>
       </c>
@@ -5589,7 +5620,7 @@
         <v>8.3079279305312733E-5</v>
       </c>
     </row>
-    <row r="126" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E126" t="s">
         <v>14</v>
       </c>
@@ -5603,7 +5634,7 @@
         <v>6.86307089913453E-5</v>
       </c>
     </row>
-    <row r="127" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E127" t="s">
         <v>3</v>
       </c>
@@ -5617,7 +5648,7 @@
         <v>6.86307089913453E-5</v>
       </c>
     </row>
-    <row r="128" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E128" t="s">
         <v>8</v>
       </c>
@@ -5631,7 +5662,7 @@
         <v>6.5018566412853448E-5</v>
       </c>
     </row>
-    <row r="129" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E129" t="s">
         <v>3</v>
       </c>
@@ -5645,7 +5676,7 @@
         <v>6.5018566412853448E-5</v>
       </c>
     </row>
-    <row r="130" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E130" t="s">
         <v>3</v>
       </c>
@@ -5659,7 +5690,7 @@
         <v>5.7794281255869725E-5</v>
       </c>
     </row>
-    <row r="131" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E131" t="s">
         <v>4</v>
       </c>
@@ -5673,7 +5704,7 @@
         <v>5.418213867737788E-5</v>
       </c>
     </row>
-    <row r="132" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E132" t="s">
         <v>9</v>
       </c>
@@ -5687,7 +5718,7 @@
         <v>5.418213867737788E-5</v>
       </c>
     </row>
-    <row r="133" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E133" t="s">
         <v>6</v>
       </c>
@@ -5701,7 +5732,7 @@
         <v>5.418213867737788E-5</v>
       </c>
     </row>
-    <row r="134" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E134" t="s">
         <v>14</v>
       </c>
@@ -5715,7 +5746,7 @@
         <v>4.6957853520394157E-5</v>
       </c>
     </row>
-    <row r="135" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E135" t="s">
         <v>15</v>
       </c>
@@ -5729,7 +5760,7 @@
         <v>3.9733568363410441E-5</v>
       </c>
     </row>
-    <row r="136" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E136" t="s">
         <v>10</v>
       </c>
@@ -5743,7 +5774,7 @@
         <v>3.6121425784918582E-5</v>
       </c>
     </row>
-    <row r="137" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E137" t="s">
         <v>17</v>
       </c>
@@ -5757,7 +5788,7 @@
         <v>3.2509283206426724E-5</v>
       </c>
     </row>
-    <row r="138" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="138" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E138" t="s">
         <v>3</v>
       </c>
@@ -5771,7 +5802,7 @@
         <v>2.8897140627934863E-5</v>
       </c>
     </row>
-    <row r="139" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E139" t="s">
         <v>3</v>
       </c>
@@ -5785,7 +5816,7 @@
         <v>2.5284998049443008E-5</v>
       </c>
     </row>
-    <row r="140" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E140" t="s">
         <v>14</v>
       </c>
@@ -5799,7 +5830,7 @@
         <v>2.1672855470951149E-5</v>
       </c>
     </row>
-    <row r="141" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E141" t="s">
         <v>3</v>
       </c>
@@ -5813,7 +5844,7 @@
         <v>2.1672855470951149E-5</v>
       </c>
     </row>
-    <row r="142" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E142" t="s">
         <v>3</v>
       </c>
@@ -5827,7 +5858,7 @@
         <v>2.1672855470951149E-5</v>
       </c>
     </row>
-    <row r="143" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="143" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E143" t="s">
         <v>15</v>
       </c>
@@ -5841,7 +5872,7 @@
         <v>2.1672855470951149E-5</v>
       </c>
     </row>
-    <row r="144" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E144" t="s">
         <v>15</v>
       </c>
@@ -5855,7 +5886,7 @@
         <v>2.1672855470951149E-5</v>
       </c>
     </row>
-    <row r="145" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E145" t="s">
         <v>10</v>
       </c>
@@ -5869,7 +5900,7 @@
         <v>1.4448570313967431E-5</v>
       </c>
     </row>
-    <row r="146" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E146" t="s">
         <v>10</v>
       </c>
@@ -5883,7 +5914,7 @@
         <v>1.4448570313967431E-5</v>
       </c>
     </row>
-    <row r="147" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E147" t="s">
         <v>3</v>
       </c>
@@ -5897,7 +5928,7 @@
         <v>1.4448570313967431E-5</v>
       </c>
     </row>
-    <row r="148" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E148" t="s">
         <v>15</v>
       </c>
@@ -5911,7 +5942,7 @@
         <v>1.4448570313967431E-5</v>
       </c>
     </row>
-    <row r="149" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E149" t="s">
         <v>10</v>
       </c>
@@ -5925,7 +5956,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="150" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E150" t="s">
         <v>20</v>
       </c>
@@ -5939,7 +5970,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="151" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E151" t="s">
         <v>3</v>
       </c>
@@ -5953,7 +5984,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="152" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E152" t="s">
         <v>3</v>
       </c>
@@ -5967,7 +5998,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="153" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E153" t="s">
         <v>3</v>
       </c>
@@ -5981,7 +6012,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="154" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E154" t="s">
         <v>15</v>
       </c>
@@ -5995,7 +6026,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="155" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E155" t="s">
         <v>15</v>
       </c>
@@ -6009,7 +6040,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="156" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E156" t="s">
         <v>15</v>
       </c>
@@ -6023,7 +6054,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="157" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E157" t="s">
         <v>15</v>
       </c>
@@ -6037,7 +6068,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="158" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E158" t="s">
         <v>15</v>
       </c>
@@ -6051,7 +6082,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="159" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E159" t="s">
         <v>16</v>
       </c>
@@ -6065,7 +6096,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="160" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E160" t="s">
         <v>19</v>
       </c>
@@ -6079,7 +6110,7 @@
         <v>1.0836427735475575E-5</v>
       </c>
     </row>
-    <row r="161" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E161" t="s">
         <v>10</v>
       </c>
@@ -6093,7 +6124,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="162" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="162" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E162" t="s">
         <v>18</v>
       </c>
@@ -6107,7 +6138,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="163" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E163" t="s">
         <v>18</v>
       </c>
@@ -6121,7 +6152,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="164" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E164" t="s">
         <v>20</v>
       </c>
@@ -6135,7 +6166,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="165" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E165" t="s">
         <v>20</v>
       </c>
@@ -6149,7 +6180,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="166" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
         <v>12</v>
       </c>
@@ -6163,7 +6194,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="167" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E167" t="s">
         <v>3</v>
       </c>
@@ -6177,7 +6208,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="168" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E168" t="s">
         <v>15</v>
       </c>
@@ -6191,7 +6222,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="169" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E169" t="s">
         <v>15</v>
       </c>
@@ -6205,7 +6236,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="170" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E170" t="s">
         <v>15</v>
       </c>
@@ -6219,7 +6250,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="171" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E171" t="s">
         <v>7</v>
       </c>
@@ -6233,7 +6264,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="172" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E172" t="s">
         <v>7</v>
       </c>
@@ -6247,7 +6278,7 @@
         <v>7.2242851569837156E-6</v>
       </c>
     </row>
-    <row r="173" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E173" t="s">
         <v>14</v>
       </c>
@@ -6261,7 +6292,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="174" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E174" t="s">
         <v>14</v>
       </c>
@@ -6275,7 +6306,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="175" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E175" t="s">
         <v>10</v>
       </c>
@@ -6289,7 +6320,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="176" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E176" t="s">
         <v>10</v>
       </c>
@@ -6303,7 +6334,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="177" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E177" t="s">
         <v>10</v>
       </c>
@@ -6317,7 +6348,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="178" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E178" t="s">
         <v>4</v>
       </c>
@@ -6331,7 +6362,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="179" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E179" t="s">
         <v>4</v>
       </c>
@@ -6345,7 +6376,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="180" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E180" t="s">
         <v>4</v>
       </c>
@@ -6359,7 +6390,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="181" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E181" t="s">
         <v>4</v>
       </c>
@@ -6373,7 +6404,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="182" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E182" t="s">
         <v>18</v>
       </c>
@@ -6387,7 +6418,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="183" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E183" t="s">
         <v>20</v>
       </c>
@@ -6401,7 +6432,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="184" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E184" t="s">
         <v>20</v>
       </c>
@@ -6415,7 +6446,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="185" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E185" t="s">
         <v>20</v>
       </c>
@@ -6429,7 +6460,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="186" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E186" t="s">
         <v>21</v>
       </c>
@@ -6443,7 +6474,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="187" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="187" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E187" t="s">
         <v>8</v>
       </c>
@@ -6457,7 +6488,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="188" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E188" t="s">
         <v>8</v>
       </c>
@@ -6471,7 +6502,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="189" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E189" t="s">
         <v>8</v>
       </c>
@@ -6485,7 +6516,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="190" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="190" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E190" t="s">
         <v>12</v>
       </c>
@@ -6499,7 +6530,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="191" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="191" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E191" t="s">
         <v>3</v>
       </c>
@@ -6513,7 +6544,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="192" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="192" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E192" t="s">
         <v>3</v>
       </c>
@@ -6527,7 +6558,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="193" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E193" t="s">
         <v>3</v>
       </c>
@@ -6541,7 +6572,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="194" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E194" t="s">
         <v>3</v>
       </c>
@@ -6555,7 +6586,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="195" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E195" t="s">
         <v>3</v>
       </c>
@@ -6569,7 +6600,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="196" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E196" t="s">
         <v>3</v>
       </c>
@@ -6583,7 +6614,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="197" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E197" t="s">
         <v>3</v>
       </c>
@@ -6597,7 +6628,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="198" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E198" t="s">
         <v>3</v>
       </c>
@@ -6611,7 +6642,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="199" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E199" t="s">
         <v>3</v>
       </c>
@@ -6625,7 +6656,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="200" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E200" t="s">
         <v>15</v>
       </c>
@@ -6639,7 +6670,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="201" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E201" t="s">
         <v>15</v>
       </c>
@@ -6653,7 +6684,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="202" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="202" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E202" t="s">
         <v>15</v>
       </c>
@@ -6667,7 +6698,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="203" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="203" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E203" t="s">
         <v>15</v>
       </c>
@@ -6681,7 +6712,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="204" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="204" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E204" t="s">
         <v>15</v>
       </c>
@@ -6695,7 +6726,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="205" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="205" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E205" t="s">
         <v>15</v>
       </c>
@@ -6709,7 +6740,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="206" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="206" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E206" t="s">
         <v>15</v>
       </c>
@@ -6723,7 +6754,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="207" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="207" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E207" t="s">
         <v>7</v>
       </c>
@@ -6737,7 +6768,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="208" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="208" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E208" t="s">
         <v>7</v>
       </c>
@@ -6751,7 +6782,7 @@
         <v>3.6121425784918578E-6</v>
       </c>
     </row>
-    <row r="209" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="209" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E209" t="s">
         <v>6</v>
       </c>
@@ -6773,18 +6804,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7CCD008-3B8B-4B6D-9F11-14C28298581D}">
   <dimension ref="A1:H78"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6807,7 +6838,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -6830,7 +6861,7 @@
         <v>0.16116371287529335</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -6853,7 +6884,7 @@
         <v>0.15566075908392005</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -6876,7 +6907,7 @@
         <v>0.13955652666504814</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -6899,7 +6930,7 @@
         <v>0.10466941814356236</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -6922,7 +6953,7 @@
         <v>8.1346605163065466E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -6945,7 +6976,7 @@
         <v>3.9111434814275307E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -6968,7 +6999,7 @@
         <v>3.0144857165978797E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -6991,7 +7022,7 @@
         <v>2.3743627093954844E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -7014,7 +7045,7 @@
         <v>2.2618758598365298E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -7037,7 +7068,7 @@
         <v>1.9260338269806589E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -7060,7 +7091,7 @@
         <v>1.811119203690216E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -7083,7 +7114,7 @@
         <v>1.7455693129400339E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -7106,7 +7137,7 @@
         <v>1.6953953224892772E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -7129,7 +7160,7 @@
         <v>1.6071862102452053E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -7152,7 +7183,7 @@
         <v>1.5068382293436919E-2</v>
       </c>
     </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>4</v>
       </c>
@@ -7166,7 +7197,7 @@
         <v>1.4162013433681312E-2</v>
       </c>
     </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>7</v>
       </c>
@@ -7180,7 +7211,7 @@
         <v>1.0633648943918429E-2</v>
       </c>
     </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>4</v>
       </c>
@@ -7194,7 +7225,7 @@
         <v>9.3792991826495108E-3</v>
       </c>
     </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>4</v>
       </c>
@@ -7208,7 +7239,7 @@
         <v>9.160799546815571E-3</v>
       </c>
     </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>4</v>
       </c>
@@ -7222,7 +7253,7 @@
         <v>8.4567451646839851E-3</v>
       </c>
     </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
         <v>8</v>
       </c>
@@ -7236,7 +7267,7 @@
         <v>8.2220603706401225E-3</v>
       </c>
     </row>
-    <row r="23" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
         <v>3</v>
       </c>
@@ -7250,7 +7281,7 @@
         <v>7.4370801974589298E-3</v>
       </c>
     </row>
-    <row r="24" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
         <v>11</v>
       </c>
@@ -7264,7 +7295,7 @@
         <v>6.3122117018693854E-3</v>
       </c>
     </row>
-    <row r="25" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
         <v>8</v>
       </c>
@@ -7278,7 +7309,7 @@
         <v>5.1145099943351946E-3</v>
       </c>
     </row>
-    <row r="26" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
         <v>4</v>
       </c>
@@ -7292,7 +7323,7 @@
         <v>4.9121955167111759E-3</v>
       </c>
     </row>
-    <row r="27" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E27" t="s">
         <v>10</v>
       </c>
@@ -7306,7 +7337,7 @@
         <v>4.5318442987780207E-3</v>
       </c>
     </row>
-    <row r="28" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E28" t="s">
         <v>12</v>
       </c>
@@ -7320,7 +7351,7 @@
         <v>4.4266407704135306E-3</v>
       </c>
     </row>
-    <row r="29" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E29" t="s">
         <v>21</v>
       </c>
@@ -7334,7 +7365,7 @@
         <v>4.1514930808448655E-3</v>
       </c>
     </row>
-    <row r="30" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E30" t="s">
         <v>3</v>
       </c>
@@ -7348,7 +7379,7 @@
         <v>3.9410860241158854E-3</v>
       </c>
     </row>
-    <row r="31" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E31" t="s">
         <v>4</v>
       </c>
@@ -7362,7 +7393,7 @@
         <v>3.7468641255968276E-3</v>
       </c>
     </row>
-    <row r="32" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
         <v>13</v>
       </c>
@@ -7376,7 +7407,7 @@
         <v>2.9537913733106739E-3</v>
       </c>
     </row>
-    <row r="33" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E33" t="s">
         <v>4</v>
       </c>
@@ -7390,7 +7421,7 @@
         <v>2.9376062151007525E-3</v>
       </c>
     </row>
-    <row r="34" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E34" t="s">
         <v>9</v>
       </c>
@@ -7404,7 +7435,7 @@
         <v>2.5815327344824797E-3</v>
       </c>
     </row>
-    <row r="35" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E35" t="s">
         <v>4</v>
       </c>
@@ -7418,7 +7449,7 @@
         <v>2.5410698389576759E-3</v>
       </c>
     </row>
-    <row r="36" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E36" t="s">
         <v>3</v>
       </c>
@@ -7432,7 +7463,7 @@
         <v>2.2901998867038927E-3</v>
       </c>
     </row>
-    <row r="37" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
         <v>4</v>
       </c>
@@ -7446,7 +7477,7 @@
         <v>2.1849963583394027E-3</v>
       </c>
     </row>
-    <row r="38" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E38" t="s">
         <v>12</v>
       </c>
@@ -7460,7 +7491,7 @@
         <v>2.1607186210245207E-3</v>
       </c>
     </row>
-    <row r="39" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E39" t="s">
         <v>3</v>
       </c>
@@ -7474,7 +7505,7 @@
         <v>1.8774783523508943E-3</v>
       </c>
     </row>
-    <row r="40" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E40" t="s">
         <v>6</v>
       </c>
@@ -7488,7 +7519,7 @@
         <v>1.658978716516954E-3</v>
       </c>
     </row>
-    <row r="41" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E41" t="s">
         <v>6</v>
       </c>
@@ -7502,7 +7533,7 @@
         <v>1.6427935583070324E-3</v>
       </c>
     </row>
-    <row r="42" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>4</v>
       </c>
@@ -7516,7 +7547,7 @@
         <v>1.5780529254673463E-3</v>
       </c>
     </row>
-    <row r="43" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>4</v>
       </c>
@@ -7530,7 +7561,7 @@
         <v>1.1329610746945052E-3</v>
       </c>
     </row>
-    <row r="44" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>4</v>
       </c>
@@ -7544,7 +7575,7 @@
         <v>1.0844056000647406E-3</v>
       </c>
     </row>
-    <row r="45" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
         <v>4</v>
       </c>
@@ -7558,7 +7589,7 @@
         <v>1.043942704539937E-3</v>
       </c>
     </row>
-    <row r="46" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
         <v>9</v>
       </c>
@@ -7572,7 +7603,7 @@
         <v>7.2833211944646763E-4</v>
       </c>
     </row>
-    <row r="47" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
         <v>14</v>
       </c>
@@ -7586,7 +7617,7 @@
         <v>6.7977664481670306E-4</v>
       </c>
     </row>
-    <row r="48" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
         <v>19</v>
       </c>
@@ -7600,7 +7631,7 @@
         <v>5.3411022092740958E-4</v>
       </c>
     </row>
-    <row r="49" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>4</v>
       </c>
@@ -7614,7 +7645,7 @@
         <v>4.8555474629764507E-4</v>
       </c>
     </row>
-    <row r="50" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>4</v>
       </c>
@@ -7628,7 +7659,7 @@
         <v>4.7746216719268429E-4</v>
       </c>
     </row>
-    <row r="51" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>6</v>
       </c>
@@ -7642,7 +7673,7 @@
         <v>4.6127700898276278E-4</v>
       </c>
     </row>
-    <row r="52" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>6</v>
       </c>
@@ -7656,7 +7687,7 @@
         <v>4.5318442987780206E-4</v>
       </c>
     </row>
-    <row r="53" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>4</v>
       </c>
@@ -7670,7 +7701,7 @@
         <v>4.4509185077284128E-4</v>
       </c>
     </row>
-    <row r="54" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>4</v>
       </c>
@@ -7684,7 +7715,7 @@
         <v>3.6416605972323381E-4</v>
       </c>
     </row>
-    <row r="55" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>6</v>
       </c>
@@ -7698,7 +7729,7 @@
         <v>3.6416605972323381E-4</v>
       </c>
     </row>
-    <row r="56" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>4</v>
       </c>
@@ -7712,7 +7743,7 @@
         <v>3.5607348061827304E-4</v>
       </c>
     </row>
-    <row r="57" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>6</v>
       </c>
@@ -7726,7 +7757,7 @@
         <v>2.9133284777858702E-4</v>
       </c>
     </row>
-    <row r="58" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>4</v>
       </c>
@@ -7740,7 +7771,7 @@
         <v>1.9422189851905802E-4</v>
       </c>
     </row>
-    <row r="59" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E59" t="s">
         <v>4</v>
       </c>
@@ -7754,7 +7785,7 @@
         <v>1.6185158209921501E-4</v>
       </c>
     </row>
-    <row r="60" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E60" t="s">
         <v>3</v>
       </c>
@@ -7768,7 +7799,7 @@
         <v>1.5375900299425426E-4</v>
       </c>
     </row>
-    <row r="61" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
         <v>8</v>
       </c>
@@ -7782,7 +7813,7 @@
         <v>1.3757384478433276E-4</v>
       </c>
     </row>
-    <row r="62" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
         <v>3</v>
       </c>
@@ -7796,7 +7827,7 @@
         <v>8.0925791049607507E-5</v>
       </c>
     </row>
-    <row r="63" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
         <v>12</v>
       </c>
@@ -7810,7 +7841,7 @@
         <v>7.2833211944646755E-5</v>
       </c>
     </row>
-    <row r="64" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E64" t="s">
         <v>7</v>
       </c>
@@ -7824,7 +7855,7 @@
         <v>6.4740632839686003E-5</v>
       </c>
     </row>
-    <row r="65" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
         <v>9</v>
       </c>
@@ -7838,7 +7869,7 @@
         <v>4.8555474629764505E-5</v>
       </c>
     </row>
-    <row r="66" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
         <v>6</v>
       </c>
@@ -7852,7 +7883,7 @@
         <v>4.8555474629764505E-5</v>
       </c>
     </row>
-    <row r="67" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
         <v>6</v>
       </c>
@@ -7866,7 +7897,7 @@
         <v>4.8555474629764505E-5</v>
       </c>
     </row>
-    <row r="68" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
         <v>11</v>
       </c>
@@ -7880,7 +7911,7 @@
         <v>3.2370316419843001E-5</v>
       </c>
     </row>
-    <row r="69" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E69" t="s">
         <v>6</v>
       </c>
@@ -7894,7 +7925,7 @@
         <v>2.4277737314882253E-5</v>
       </c>
     </row>
-    <row r="70" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E70" t="s">
         <v>10</v>
       </c>
@@ -7908,7 +7939,7 @@
         <v>1.6185158209921501E-5</v>
       </c>
     </row>
-    <row r="71" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E71" t="s">
         <v>4</v>
       </c>
@@ -7922,7 +7953,7 @@
         <v>1.6185158209921501E-5</v>
       </c>
     </row>
-    <row r="72" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E72" t="s">
         <v>9</v>
       </c>
@@ -7936,7 +7967,7 @@
         <v>1.6185158209921501E-5</v>
       </c>
     </row>
-    <row r="73" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
         <v>14</v>
       </c>
@@ -7950,7 +7981,7 @@
         <v>8.0925791049607503E-6</v>
       </c>
     </row>
-    <row r="74" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
         <v>5</v>
       </c>
@@ -7964,7 +7995,7 @@
         <v>8.0925791049607503E-6</v>
       </c>
     </row>
-    <row r="75" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E75" t="s">
         <v>4</v>
       </c>
@@ -7978,7 +8009,7 @@
         <v>8.0925791049607503E-6</v>
       </c>
     </row>
-    <row r="76" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E76" t="s">
         <v>9</v>
       </c>
@@ -7992,7 +8023,7 @@
         <v>8.0925791049607503E-6</v>
       </c>
     </row>
-    <row r="77" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>9</v>
       </c>
@@ -8006,7 +8037,7 @@
         <v>8.0925791049607503E-6</v>
       </c>
     </row>
-    <row r="78" spans="5:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="5:8" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
         <v>8</v>
       </c>

</xml_diff>